<commit_message>
Revert "Sync from main"
</commit_message>
<xml_diff>
--- a/data/explorer_outputs.xlsx
+++ b/data/explorer_outputs.xlsx
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K11"/>
+  <dimension ref="A1:K10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1015,61 +1015,6 @@
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>2026-06-16T18:03:06</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>openai</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>gpt-5.5</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Find stocks where the LLV is 2 times lower than the HHV, RSI is below 20 and close is above 20 day moving average</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>LLV Half HHV RSI MA</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>Finds stocks where the 20-period lowest low is at most half of the 20-period highest high, RSI(14) is below 20, and the close is above the 20-day simple moving average. Assumes LLV uses L, HHV uses H, RSI defaults to 14 periods, and moving average defaults to simple.</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>LLV(L,20) &lt;= HHV(H,20) / 2 AND RSI(14) &lt; 20 AND C &gt; Mov(C,20,S)</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>[{"col_letter": "A", "col_code": "LLV(L,20)"}, {"col_letter": "B", "col_code": "HHV(H,20)"}, {"col_letter": "C", "col_code": "RSI(14)"}, {"col_letter": "D", "col_code": "C"}, {"col_letter": "E", "col_code": "Mov(C,20,S)"}]</t>
-        </is>
-      </c>
-      <c r="I11" t="b">
-        <v>1</v>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>{"explorer_name": "LLV Half HHV RSI MA", "explorer_description": "Finds stocks where the 20-period lowest low is at most half of the 20-period highest high, RSI(14) is below 20, and the close is above the 20-day simple moving average. Assumes LLV uses L, HHV uses H, RSI defaults to 14 periods, and moving average defaults to simple.", "explorer_code_body": "LLV(L,20) &lt;= HHV(H,20) / 2 AND RSI(14) &lt; 20 AND C &gt; Mov(C,20,S)", "col_definitions": [{"col_letter": "A", "col_code": "LLV(L,20)"}, {"col_letter": "B", "col_code": "HHV(H,20)"}, {"col_letter": "C", "col_code": "RSI(14)"}, {"col_letter": "D", "col_code": "C"}, {"col_letter": "E", "col_code": "Mov(C,20,S)"}]}</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>